<commit_message>
v0.83.13 — Update Docs and Keymapper
</commit_message>
<xml_diff>
--- a/remotes/keymapper/astrion/KeyCodes Astrion.xlsx
+++ b/remotes/keymapper/astrion/KeyCodes Astrion.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -841,33 +841,33 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>F1 long-press</t>
+          <t>Channel Up long-press</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>131</v>
+        <v>92</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>KEYCODE_F1</t>
+          <t>KEYCODE_PAGE_UP</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>59</v>
+        <v>104</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Android Go home</t>
+          <t>'</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>75</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>KEYCODE_APOSTROPHE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -879,33 +879,33 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>F2 long-press</t>
+          <t>Channel Down long-press</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>132</v>
+        <v>93</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>KEYCODE_F2</t>
+          <t>KEYCODE_PAGE_DOWN</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>60</v>
+        <v>109</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>=</t>
+          <t>/</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>KEYCODE_EQUALS</t>
+          <t>KEYCODE_SLASH</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -917,36 +917,112 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>F1 long-press</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>131</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>KEYCODE_F1</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>59</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Android Go home</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>group “FullyKiosk” — Fully Kiosk Browser in foreground</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>F2 long-press</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>132</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>KEYCODE_F2</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>60</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>KEYCODE_EQUALS</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>group “FullyKiosk” — Fully Kiosk Browser in foreground</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>F11 long-press</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B16" t="n">
         <v>141</v>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>KEYCODE_F11</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D16" t="n">
         <v>87</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Open Android Browser</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>com.android.browser</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>global</t>
         </is>

</xml_diff>

<commit_message>
v0.84.1 - beta release candidate
</commit_message>
<xml_diff>
--- a/remotes/keymapper/astrion/KeyCodes Astrion.xlsx
+++ b/remotes/keymapper/astrion/KeyCodes Astrion.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -841,33 +841,33 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Channel Up long-press</t>
+          <t>D-pad Left long-press</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>92</v>
+        <v>21</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>KEYCODE_PAGE_UP</t>
+          <t>KEYCODE_DPAD_LEFT</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>'</t>
+          <t>,</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>55</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>KEYCODE_APOSTROPHE</t>
+          <t>KEYCODE_COMMA</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -879,33 +879,33 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Channel Down long-press</t>
+          <t>D-pad Right long-press</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>93</v>
+        <v>22</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>KEYCODE_PAGE_DOWN</t>
+          <t>KEYCODE_DPAD_RIGHT</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>56</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>KEYCODE_SLASH</t>
+          <t>KEYCODE_PERIOD</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -917,33 +917,33 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>F1 long-press</t>
+          <t>Channel Up long-press</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>131</v>
+        <v>92</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>KEYCODE_F1</t>
+          <t>KEYCODE_PAGE_UP</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>59</v>
+        <v>104</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Android Go home</t>
+          <t>'</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>75</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>KEYCODE_APOSTROPHE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -955,33 +955,33 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>F2 long-press</t>
+          <t>Channel Down long-press</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>132</v>
+        <v>93</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>KEYCODE_F2</t>
+          <t>KEYCODE_PAGE_DOWN</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>60</v>
+        <v>109</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>=</t>
+          <t>/</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>KEYCODE_EQUALS</t>
+          <t>KEYCODE_SLASH</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -993,36 +993,112 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>F1 long-press</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>131</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>KEYCODE_F1</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>59</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Android Go home</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>group “FullyKiosk” — Fully Kiosk Browser in foreground</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>F2 long-press</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>132</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>KEYCODE_F2</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>60</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>KEYCODE_EQUALS</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>group “FullyKiosk” — Fully Kiosk Browser in foreground</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>F11 long-press</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B18" t="n">
         <v>141</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>KEYCODE_F11</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D18" t="n">
         <v>87</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Open Android Browser</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>com.android.browser</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>global</t>
         </is>

</xml_diff>